<commit_message>
Publish Szeged_2025_WC, Duisburg_2018_WC, Rome_2012_MAR, Racice_2013_WC, Milan_2025_WCH, Milan_2015_WCH, Szeged_2023_WC, Rio_2016_OG, Copenhagen_2013_MAR
</commit_message>
<xml_diff>
--- a/events/Rome_2012_MAR/Rome_2012_MAR_Results.xlsx
+++ b/events/Rome_2012_MAR/Rome_2012_MAR_Results.xlsx
@@ -2493,11 +2493,6 @@
           <t>+10:23,240</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>178014</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -11886,11 +11881,6 @@
       <c r="Q165" t="inlineStr">
         <is>
           <t>+9:51,760</t>
-        </is>
-      </c>
-      <c r="R165" t="inlineStr">
-        <is>
-          <t>178014</t>
         </is>
       </c>
     </row>
@@ -25454,7 +25444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D220"/>
+  <dimension ref="A1:D219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29134,17 +29124,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>178014</t>
+          <t>47436</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Vinicius Zabot</t>
+          <t>Pál</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>SANTOS</t>
+          <t>SARUDI</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -29156,17 +29146,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>47436</t>
+          <t>54736</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Pál</t>
+          <t>Conrad Robin</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>SARUDI</t>
+          <t>SCHEIBNER</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -29178,17 +29168,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>54736</t>
+          <t>49656</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Conrad Robin</t>
+          <t>Richárd</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>SCHEIBNER</t>
+          <t>SCHMIDT</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -29200,17 +29190,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>49656</t>
+          <t>42513</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Richárd</t>
+          <t>David</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>SCHMIDT</t>
+          <t>SCHMUDE</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -29222,39 +29212,39 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>42513</t>
+          <t>48740</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Kerry</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>SCHMUDE</t>
+          <t>SEGAL</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>48740</t>
+          <t>49765</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Kerry</t>
+          <t>Julia</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>SEGAL</t>
+          <t>SEGER</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -29266,39 +29256,39 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>49765</t>
+          <t>52283</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Julia</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>SEGER</t>
+          <t>SEIDL</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>52283</t>
+          <t>46397</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Eduard</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>SEIDL</t>
+          <t>SHEMETYLO</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -29310,17 +29300,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>46397</t>
+          <t>57969</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Eduard</t>
+          <t>Oleksii</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>SHEMETYLO</t>
+          <t>SHPAK</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -29332,17 +29322,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>57969</t>
+          <t>88454</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Oleksii</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>SHPAK</t>
+          <t>SIMMONS</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -29354,61 +29344,61 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>88454</t>
+          <t>42963</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Jonathan</t>
+          <t>Rebeka</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>SIMMONS</t>
+          <t>SIMON</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>42963</t>
+          <t>100153</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Rebeka</t>
+          <t>Ajit</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>SIMON</t>
+          <t>SINGH</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>100153</t>
+          <t>89760</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Ajit</t>
+          <t>Oleksandr</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>SINGH</t>
+          <t>SIVKOV</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -29420,17 +29410,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>89760</t>
+          <t>42376</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Oleksandr</t>
+          <t>Radek</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>SIVKOV</t>
+          <t>SLOUF</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -29442,61 +29432,61 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>42376</t>
+          <t>48778</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Kjinta</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>SLOUF</t>
+          <t>SMALLE</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>48778</t>
+          <t>49447</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Kjinta</t>
+          <t>Pablo</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>SMALLE</t>
+          <t>SOLARES</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>49447</t>
+          <t>63449</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Pablo</t>
+          <t>Timothy</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>SOLARES</t>
+          <t>STENLAKE</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -29508,61 +29498,61 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>63449</t>
+          <t>47622</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Timothy</t>
+          <t>Linnea</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>STENLAKE</t>
+          <t>STENSILS</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>47622</t>
+          <t>49751</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Linnea</t>
+          <t>Emil</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>STENSILS</t>
+          <t>SVENSSON</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>49751</t>
+          <t>42599</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Emil</t>
+          <t>Grzegorz</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>SVENSSON</t>
+          <t>SZPYNDA</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -29574,17 +29564,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>42599</t>
+          <t>57974</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Grzegorz</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>SZPYNDA</t>
+          <t>SÁNCHEZ</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -29596,12 +29586,12 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>57974</t>
+          <t>57970</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Alejandro</t>
+          <t>José Manuel</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -29618,17 +29608,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>57970</t>
+          <t>50167</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>José Manuel</t>
+          <t>Carlo</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>SÁNCHEZ</t>
+          <t>TACCHINI</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -29640,39 +29630,39 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>50167</t>
+          <t>45120</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Carlo</t>
+          <t>Tamara</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>TACCHINI</t>
+          <t>TAKÁCS</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>45120</t>
+          <t>48780</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Tamara</t>
+          <t>Lisane</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>TAKÁCS</t>
+          <t>TERRIE</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -29684,17 +29674,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>48780</t>
+          <t>42349</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Lisane</t>
+          <t>Amalie</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>TERRIE</t>
+          <t>THOMSEN</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -29706,39 +29696,39 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>42349</t>
+          <t>36184</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Amalie</t>
+          <t>Leonid</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>THOMSEN</t>
+          <t>TILSH</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>36184</t>
+          <t>61292</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Leonid</t>
+          <t>Malin</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>TILSH</t>
+          <t>TITORIC</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -29750,17 +29740,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>61292</t>
+          <t>49762</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Malin</t>
+          <t>Emil</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>TITORIC</t>
+          <t>TORSTENSSON</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -29772,17 +29762,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>49762</t>
+          <t>48841</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Emil</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>TORSTENSSON</t>
+          <t>TYE</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -29794,17 +29784,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>48841</t>
+          <t>36742</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Jonathan</t>
+          <t>Lars Magne</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>TYE</t>
+          <t>ULLVANG</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -29816,17 +29806,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>36742</t>
+          <t>35416</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Lars Magne</t>
+          <t>Quentin</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>ULLVANG</t>
+          <t>URBAN</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -29838,17 +29828,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>35416</t>
+          <t>48410</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Quentin</t>
+          <t>Brandon</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>URBAN</t>
+          <t>VAN DER WALT</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -29860,56 +29850,56 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>48410</t>
+          <t>56464</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Brandon</t>
+          <t>Ana</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>VAN DER WALT</t>
+          <t>VARELA</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>56464</t>
+          <t>47429</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Ana</t>
+          <t>Dávid</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>VARELA</t>
+          <t>VARGA</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>47429</t>
+          <t>54279</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Dávid</t>
+          <t>Patrik</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -29926,56 +29916,56 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>54279</t>
+          <t>36600</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Patrik</t>
+          <t>Oona</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>VARGA</t>
+          <t>VASKO</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>36600</t>
+          <t>63247</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Oona</t>
+          <t>Carlos</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>VASKO</t>
+          <t>VEGA</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>63247</t>
+          <t>46844</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>Miriam</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -29985,112 +29975,112 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>46844</t>
+          <t>71638</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Miriam</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>VEGA</t>
+          <t>VERDUYCKT</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>71638</t>
+          <t>49437</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Erik</t>
+          <t>Nuria</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>VERDUYCKT</t>
+          <t>VILLACE</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>49437</t>
+          <t>36586</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Nuria</t>
+          <t>Filippo</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>VILLACE</t>
+          <t>VINCENZI</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>36586</t>
+          <t>49659</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Filippo</t>
+          <t>Enikö</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>VINCENZI</t>
+          <t>VÁCZAI</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>49659</t>
+          <t>42964</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Enikö</t>
+          <t>Amy</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>VÁCZAI</t>
+          <t>WARD</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -30102,17 +30092,17 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>42964</t>
+          <t>47624</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Amy</t>
+          <t>Moa</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>WARD</t>
+          <t>WIKBERG</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -30124,34 +30114,34 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>47624</t>
+          <t>42232</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Moa</t>
+          <t>Fabio</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>WIKBERG</t>
+          <t>WYSS</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>42232</t>
+          <t>37574</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Fabio</t>
+          <t>Silvan</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -30168,61 +30158,61 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>37574</t>
+          <t>56582</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Silvan</t>
+          <t>Penelope</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>WYSS</t>
+          <t>YOUNG</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>56582</t>
+          <t>36310</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Penelope</t>
+          <t>Jost</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>YOUNG</t>
+          <t>ZAKRAJSEK</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>36310</t>
+          <t>49457</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Jost</t>
+          <t>Mateusz</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>ZAKRAJSEK</t>
+          <t>ZUCHORA</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -30234,17 +30224,17 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>49457</t>
+          <t>49443</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Mateusz</t>
+          <t>Alan</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>ZUCHORA</t>
+          <t>ÁVILA</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -30256,42 +30246,20 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>49443</t>
+          <t>49516</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Alan</t>
+          <t>David</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>ÁVILA</t>
+          <t>ÚRSULA</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>49516</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>David</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr">
-        <is>
-          <t>ÚRSULA</t>
-        </is>
-      </c>
-      <c r="D220" t="inlineStr">
         <is>
           <t>M</t>
         </is>

</xml_diff>